<commit_message>
Updated with version 2 (k=4)
</commit_message>
<xml_diff>
--- a/RAG_Version_Metrics_Tracker.xlsx
+++ b/RAG_Version_Metrics_Tracker.xlsx
@@ -41,14 +41,14 @@
 Generator: GROQ</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 2
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
+    <t>Version 2
+Chunker: Normal fix length chunkker
+Embedding Model:  BAAI/bge-small-en-v1.5
+Chunk Size: 500
+Overlap: 100
+Top K: 4  ------------
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
   </si>
   <si>
     <t xml:space="preserve">Version 3
@@ -260,7 +260,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -314,12 +314,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
@@ -329,7 +332,10 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -650,217 +656,225 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="48.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="48.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="12.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="32" customFormat="1" s="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="116.25" customFormat="1" s="1">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="5">
         <v>1</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="5">
         <v>0.9</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="5">
         <v>0.48</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="5">
         <v>0.98</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="116.25" customFormat="1" s="1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>0.98</v>
+      </c>
+      <c r="D3" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.98</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="116.25" customFormat="1" s="1">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated with version 3 metrics
</commit_message>
<xml_diff>
--- a/RAG_Version_Metrics_Tracker.xlsx
+++ b/RAG_Version_Metrics_Tracker.xlsx
@@ -51,14 +51,14 @@
 Generator: GROQ</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 3
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
+    <t>Version 3
+Chunker: Normal fix length chunkker
+Embedding Model:  BAAI/bge-small-en-v1.5
+Chunk Size: 500
+Overlap: 100
+Top K: 5  ------------
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
   </si>
   <si>
     <t xml:space="preserve">Version 4
@@ -688,13 +688,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="5">
-        <v>0.9</v>
+        <v>0.982</v>
       </c>
       <c r="D2" s="5">
-        <v>0.48</v>
+        <v>0.4</v>
       </c>
       <c r="E2" s="5">
-        <v>0.98</v>
+        <v>0.958</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="116.25" customFormat="1" s="1">
@@ -705,23 +705,31 @@
         <v>1</v>
       </c>
       <c r="C3" s="5">
-        <v>0.98</v>
+        <v>0.987</v>
       </c>
       <c r="D3" s="5">
-        <v>0.4</v>
+        <v>0.302</v>
       </c>
       <c r="E3" s="5">
-        <v>0.98</v>
+        <v>0.958</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="116.25" customFormat="1" s="1">
       <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="B4" s="5">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5">
+        <v>0.992</v>
+      </c>
+      <c r="D4" s="5">
+        <v>0.244</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0.958</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A5" s="4" t="s">

</xml_diff>

<commit_message>
Changed the structure of the evaluation metrics
</commit_message>
<xml_diff>
--- a/RAG_Version_Metrics_Tracker.xlsx
+++ b/RAG_Version_Metrics_Tracker.xlsx
@@ -36,19 +36,19 @@
 Embedding Model:  BAAI/bge-small-en-v1.5
 Chunk Size: 500
 Overlap: 100
-Top K: 3
+Top K: 3 --------- changing factor
 Retriever Method: Cosine Similarity
 Generator: GROQ</t>
   </si>
   <si>
-    <t>Version 2
+    <t xml:space="preserve">Version 2
 Chunker: Normal fix length chunkker
 Embedding Model:  BAAI/bge-small-en-v1.5
 Chunk Size: 500
 Overlap: 100
-Top K: 4  ------------
+Top K: 4  ------------  changing factor
 Retriever Method: Cosine Similarity
-Generator: GROQ</t>
+Generator: GROQ </t>
   </si>
   <si>
     <t>Version 3
@@ -56,7 +56,7 @@
 Embedding Model:  BAAI/bge-small-en-v1.5
 Chunk Size: 500
 Overlap: 100
-Top K: 5  ------------
+Top K: 5  ------------ changing factor
 Retriever Method: Cosine Similarity
 Generator: GROQ</t>
   </si>
@@ -731,7 +731,7 @@
         <v>0.958</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="120" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="116.25" customFormat="1" s="1">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Updated with Embedding metric evaluation
</commit_message>
<xml_diff>
--- a/RAG_Version_Metrics_Tracker.xlsx
+++ b/RAG_Version_Metrics_Tracker.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Versions</t>
   </si>
@@ -36,7 +36,7 @@
 Embedding Model:  BAAI/bge-small-en-v1.5
 Chunk Size: 500
 Overlap: 100
-Top K: 3 --------- changing factor
+Top K: 3 --------- (changing factor)
 Retriever Method: Cosine Similarity
 Generator: GROQ</t>
   </si>
@@ -46,7 +46,7 @@
 Embedding Model:  BAAI/bge-small-en-v1.5
 Chunk Size: 500
 Overlap: 100
-Top K: 4  ------------  changing factor
+Top K: 4  ------------  (changing factor)
 Retriever Method: Cosine Similarity
 Generator: GROQ </t>
   </si>
@@ -56,89 +56,42 @@
 Embedding Model:  BAAI/bge-small-en-v1.5
 Chunk Size: 500
 Overlap: 100
-Top K: 5  ------------ changing factor
+Top K: 5  ------------ (changing factor)
 Retriever Method: Cosine Similarity
 Generator: GROQ</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 4
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 5
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 6
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 7
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 8
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 9
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 10
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 11
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
+    <t>Version 4
+Chunker: Normal fix length chunkker
+Embedding Model:  BAAI/bge-small-en-v1.5 ---(changing factor)
+Chunk Size: 500
+Overlap: 100
+Top K: 4
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
+  </si>
+  <si>
+    <t>Version 4
+Chunker: Normal fix length chunkker
+Embedding Model:  intfloat/e5-base-v2 ---(changing factor)
+Chunk Size: 500
+Overlap: 100
+Top K: 4
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
+  </si>
+  <si>
+    <t>Version 4
+Chunker: Normal fix length chunkker
+Embedding Model:  nomic-ai/nomic-embed-text-v1.5 ---(changing factor)
+Chunk Size: 500
+Overlap: 100
+Top K: 4
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t xml:space="preserve">Version 12
@@ -314,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -330,6 +283,9 @@
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -656,11 +612,11 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="48.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="48.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="8" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="12.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="32" customFormat="1" s="1">
@@ -735,19 +691,35 @@
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>0.982</v>
+      </c>
+      <c r="D5" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E5" s="5">
+        <v>0.958</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="B6" s="5">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5">
+        <v>0.982</v>
+      </c>
+      <c r="D6" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0.958</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A7" s="4" t="s">
@@ -759,7 +731,7 @@
       <c r="E7" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="5"/>
@@ -768,8 +740,8 @@
       <c r="E8" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A9" s="4" t="s">
-        <v>12</v>
+      <c r="A9" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -777,8 +749,8 @@
       <c r="E9" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A10" s="4" t="s">
-        <v>13</v>
+      <c r="A10" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -786,8 +758,8 @@
       <c r="E10" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A11" s="4" t="s">
-        <v>14</v>
+      <c r="A11" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -795,8 +767,8 @@
       <c r="E11" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A12" s="4" t="s">
-        <v>15</v>
+      <c r="A12" s="6" t="s">
+        <v>11</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -805,7 +777,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A13" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -814,7 +786,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A14" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -823,7 +795,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A15" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -832,7 +804,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A16" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -841,7 +813,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A17" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -850,7 +822,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A18" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -859,7 +831,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A19" s="4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -868,7 +840,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A20" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -877,7 +849,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="120" customFormat="1" s="1">
       <c r="A21" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>

</xml_diff>

<commit_message>
Done with chunk size and overlap experimenting
</commit_message>
<xml_diff>
--- a/RAG_Version_Metrics_Tracker.xlsx
+++ b/RAG_Version_Metrics_Tracker.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
   <si>
     <t>Versions</t>
   </si>
@@ -71,7 +71,7 @@
 Generator: GROQ</t>
   </si>
   <si>
-    <t>Version 4
+    <t>Version 5
 Chunker: Normal fix length chunkker
 Embedding Model:  intfloat/e5-base-v2 ---(changing factor)
 Chunk Size: 500
@@ -81,7 +81,7 @@
 Generator: GROQ</t>
   </si>
   <si>
-    <t>Version 4
+    <t>Version 6
 Chunker: Normal fix length chunkker
 Embedding Model:  nomic-ai/nomic-embed-text-v1.5 ---(changing factor)
 Chunk Size: 500
@@ -91,97 +91,47 @@
 Generator: GROQ</t>
   </si>
   <si>
+    <t>Version 7
+Chunker: Normal fix length chunkker
+Embedding Model:  BAAI/bge-small-en-v1.5
+Chunk Size: 500 --------- (changing factor)
+Overlap: 100 --------- (changing factor)
+Top K: 3 
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
+  </si>
+  <si>
+    <t>Version 8
+Chunker: Normal fix length chunkker
+Embedding Model:  BAAI/bge-small-en-v1.5
+Chunk Size: 300 --------- (changing factor)
+Overlap: 60 --------- (changing factor)
+Top K: 3 
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
+  </si>
+  <si>
+    <t>Version 9
+Chunker: Normal fix length chunkker
+Embedding Model:  BAAI/bge-small-en-v1.5
+Chunk Size: 700 --------- (changing factor)
+Overlap: 100 --------- (changing factor)
+Top K: 3 
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
+  </si>
+  <si>
+    <t>Version 10
+Chunker: Normal fix length chunkker
+Embedding Model:  BAAI/bge-small-en-v1.5
+Chunk Size: 500 --------- (changing factor)
+Overlap: 50 --------- (changing factor)
+Top K: 3 
+Retriever Method: Cosine Similarity
+Generator: GROQ</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 12
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 13
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 14
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 15
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 16
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 17
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 18
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 19
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Version 20
-Chunker: 
-Embedding Model: 
-Chunk Size: 
-Overlap: 
-Top K: 
-Retriever Method: 
-Generator: </t>
   </si>
 </sst>
 </file>
@@ -739,44 +689,76 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A10" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="120" customFormat="1" s="1">
+      <c r="B8" s="5">
+        <v>1</v>
+      </c>
+      <c r="C8" s="5">
+        <v>0.987</v>
+      </c>
+      <c r="D8" s="5">
+        <v>0.302</v>
+      </c>
+      <c r="E8" s="5">
+        <v>0.958</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="116.25" customFormat="1" s="1">
+      <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="5">
+        <v>1</v>
+      </c>
+      <c r="C9" s="5">
+        <v>0.744</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0.522</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="116.25" customFormat="1" s="1">
+      <c r="A10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="5">
+        <v>1</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0.866</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0.43</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0.973</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="116.25" customFormat="1" s="1">
+      <c r="A11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="5">
+        <v>1</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.854</v>
+      </c>
+      <c r="D11" s="5">
+        <v>0.42</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0.968</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A12" s="6" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -784,8 +766,8 @@
       <c r="E12" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A13" s="4" t="s">
-        <v>12</v>
+      <c r="A13" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -793,8 +775,8 @@
       <c r="E13" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A14" s="4" t="s">
-        <v>13</v>
+      <c r="A14" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -802,8 +784,8 @@
       <c r="E14" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A15" s="4" t="s">
-        <v>14</v>
+      <c r="A15" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -811,7 +793,7 @@
       <c r="E15" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="5"/>
@@ -820,8 +802,8 @@
       <c r="E16" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A17" s="4" t="s">
-        <v>16</v>
+      <c r="A17" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -829,8 +811,8 @@
       <c r="E17" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A18" s="4" t="s">
-        <v>17</v>
+      <c r="A18" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -838,8 +820,8 @@
       <c r="E18" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A19" s="4" t="s">
-        <v>18</v>
+      <c r="A19" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -847,8 +829,8 @@
       <c r="E19" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A20" s="4" t="s">
-        <v>19</v>
+      <c r="A20" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -856,8 +838,8 @@
       <c r="E20" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="120" customFormat="1" s="1">
-      <c r="A21" s="4" t="s">
-        <v>20</v>
+      <c r="A21" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>

</xml_diff>